<commit_message>
new form from gaps poc
</commit_message>
<xml_diff>
--- a/modules/data/structures/storage/onboarding_clinicians.xlsx
+++ b/modules/data/structures/storage/onboarding_clinicians.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" state="visible" r:id="rId2"/>
@@ -359,7 +359,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -421,12 +421,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C11"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="57.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="57.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52.38"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="257" min="4" style="1" width="11.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="257" min="4" style="1" width="11.48"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -495,7 +495,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C30"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.69"/>
@@ -690,7 +690,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K1009"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="33.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="39.12"/>
@@ -702,7 +702,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="28.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="5" width="16.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="5" width="28.15"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="259" min="12" style="5" width="11.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="259" min="12" style="5" width="11.48"/>
   </cols>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="30.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4903,7 +4903,7 @@
       <c r="I1009" s="11"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="6">
     <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I2:I1009" type="list">
       <formula1>"Nominal,Ordinal,Discrete,Continuous,Multiple,Text"</formula1>
       <formula2>0</formula2>
@@ -4920,15 +4920,11 @@
       <formula1>"yes/no,LikertAgreement_3values,LikertAgreement_5values,LikertLikelihhod_3values,LikertLikelihood_5values,,,"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:E1 H1:AMJ1" type="none">
-      <formula1>0</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F1:F1010" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F1010" type="list">
       <formula1>",no,yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G1:G1010" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G1010" type="list">
       <formula1>",yes,no"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>